<commit_message>
fix: BOM4.ItemId tat fuzzy Tier3, chi exact/normalize - tranh mo nham du an khac
Phat hien qua Bravo: "KIEN N" (Ten kien hang, BOM4) exact match ra ma
RO.FF.02A.R... nhung ca family mo nay (~90 dong) da bi danh IsActive=false
toan bo. Nhung fuzzy Tier3 van tim ra candidate khac (vd "KIEN 1_D4" ->
2466_CT01.12.K005) - xac nhan qua ParentId=73463 la item cua 1 DU AN KHAC
hoan toan (khong lien quan SYCAMORE/DH311B dang lam), chi trung ngau nhien
tien to ten. Chon nham se gan sai san pham hoan toan.

Fix: kieu_lookup fuzzy_name -> exact_name. Tier1/2 (exact/normalize) van
giu (phong data active that khop chinh xac sau nay), nhung tat han Tier3
fuzzy - khong khop thi roi thang MKT_BB (Ma kien truc - Bao bi, dung sap
co san) nhu cach KIEN 7-10 dang hoat dong dung.

Chi sua config Excel, khong doi code.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/config/CK_Mapping_v5.xlsx
+++ b/Tools/config/CK_Mapping_v5.xlsx
@@ -7087,7 +7087,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>fuzzy_name</t>
+          <t>exact_name</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Lookup B20Item</t>
+          <t>Chi exact/normalize, tat fuzzy Tier3 - tranh mo nham sang du an khac (KIEN N la nhan lap lai, khong dinh danh on dinh). Khong khop -&gt; MKT_BB.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: thong bao/popup than thien voi end-user, bo thuat ngu ky thuat/ten bang SQL
3 cho theo dung feedback user (dua tren anh chup man hinh thuc te):

1. version.json release_notes: viet lai theo huong "cai thien gi cho cong
   viec" thay vi liet ke co che (BTP/NVL, USP, MKT, fuzzy...).

2. Popup "Cảnh báo Validator" -> "Cảnh báo trước khi Import": bo hien thi
   ten validator ky thuat (CodeUnique:). VALIDATORS sheet: WarningMessage
   cua CodeUnique dang lo thang ten bang SQL "B20BOM" ra man hinh nguoi
   dung - sua thanh cau tieng Viet binh thuong. CheckUniqueBOM cung sua
   tuong tu (bo ItemId0/Version/EffectiveDate raw).

3. Popup "Validate + DB OK" -> "Kiểm tra thành công": "mã fuzzy đã xác
   nhận" (thuat toan noi bo) -> "mã đã đối chiếu"/"mã vật tư đã được đối
   chiếu với hệ thống". Dong "0 cảnh báo" chi hien khi thuc su co canh
   bao, khong hien dong 0 vo nghia.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/config/CK_Mapping_v5.xlsx
+++ b/Tools/config/CK_Mapping_v5.xlsx
@@ -1678,7 +1678,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BOM đã tồn tại với cùng ItemId0/Version/EffectiveDate: {result}</t>
+          <t>Đã tồn tại BOM khác cùng sản phẩm, phiên bản và ngày hiệu lực: {result}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Code "{Code}" đã tồn tại trong B20BOM</t>
+          <t>Mã BOM "{Code}" đã tồn tại trong hệ thống — import lại có thể tạo bản ghi trùng.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
fix: BTP Rule 1 ap dung moi tang STT (khong chi STT nguyen) + bo sung IsTool mapping
- Rule 1 (rong + co dinh danh) gio la OR: Ten vat tu rong + (Ten chi
  tiet co gia tri HOAC co dong con ben duoi), de quy moi tang thap
  phan (1 -> 1.1 -> 1.1.1...) thay vi chi bat STT nguyen.
- Rule 2 ("+") giu nguyen, chi ap cho STT nguyen.
- Validate STT dung NUMERIC_STT_PATTERN (ho tro nhieu tang thap phan)
  thay vi replace('.', '', 1) chi dung 1 tang.
- Bump version 2.2.9 -> 2.2.10.
- CK_Mapping_v5.xlsx: bo sung field IsTool (CoDinh=1) vao HEADER.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/config/CK_Mapping_v5.xlsx
+++ b/Tools/config/CK_Mapping_v5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\insertdatasqlserver\Tools\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD41982-0913-4356-8966-67248E852309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C2DD88-44A4-428E-91F4-32BF13A45897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1780" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1784" uniqueCount="401">
   <si>
     <t>CK_Mapping_v4 — Sheet 6: HEADER — Mapping đầu phiếu (Section=HEADER → BOM | Section=THDM_HEADER → THDM)</t>
   </si>
@@ -1226,6 +1226,9 @@
   </si>
   <si>
     <t>ParentDetailRowId_SO</t>
+  </si>
+  <si>
+    <t>IsTool</t>
   </si>
 </sst>
 </file>
@@ -2489,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -3739,16 +3742,13 @@
         <v>31</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>400</v>
       </c>
       <c r="D54" t="s">
-        <v>75</v>
-      </c>
-      <c r="E54" t="s">
-        <v>82</v>
-      </c>
-      <c r="G54" t="s">
-        <v>87</v>
+        <v>52</v>
+      </c>
+      <c r="G54">
+        <v>1</v>
       </c>
       <c r="H54" t="s">
         <v>44</v>
@@ -3756,37 +3756,22 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55" t="s">
-        <v>161</v>
+        <v>31</v>
       </c>
       <c r="B55" t="s">
-        <v>140</v>
-      </c>
-      <c r="C55" t="s">
-        <v>51</v>
+        <v>160</v>
       </c>
       <c r="D55" t="s">
-        <v>52</v>
-      </c>
-      <c r="F55" t="s">
-        <v>35</v>
+        <v>75</v>
+      </c>
+      <c r="E55" t="s">
+        <v>82</v>
       </c>
       <c r="G55" t="s">
-        <v>162</v>
+        <v>87</v>
       </c>
       <c r="H55" t="s">
-        <v>54</v>
-      </c>
-      <c r="I55" t="s">
-        <v>163</v>
-      </c>
-      <c r="J55" t="s">
-        <v>69</v>
-      </c>
-      <c r="K55" t="s">
-        <v>164</v>
-      </c>
-      <c r="L55" t="s">
-        <v>165</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -3794,25 +3779,34 @@
         <v>161</v>
       </c>
       <c r="B56" t="s">
-        <v>65</v>
+        <v>140</v>
       </c>
       <c r="C56" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D56" t="s">
-        <v>166</v>
+        <v>52</v>
       </c>
       <c r="F56" t="s">
         <v>35</v>
       </c>
       <c r="G56" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="H56" t="s">
         <v>54</v>
       </c>
       <c r="I56" t="s">
-        <v>59</v>
+        <v>163</v>
+      </c>
+      <c r="J56" t="s">
+        <v>69</v>
+      </c>
+      <c r="K56" t="s">
+        <v>164</v>
+      </c>
+      <c r="L56" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -3820,7 +3814,7 @@
         <v>161</v>
       </c>
       <c r="B57" t="s">
-        <v>168</v>
+        <v>65</v>
       </c>
       <c r="C57" t="s">
         <v>57</v>
@@ -3846,22 +3840,25 @@
         <v>161</v>
       </c>
       <c r="B58" t="s">
-        <v>131</v>
+        <v>168</v>
+      </c>
+      <c r="C58" t="s">
+        <v>57</v>
       </c>
       <c r="D58" t="s">
-        <v>41</v>
-      </c>
-      <c r="E58" t="s">
-        <v>42</v>
+        <v>166</v>
       </c>
       <c r="F58" t="s">
         <v>35</v>
       </c>
       <c r="G58" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H58" t="s">
-        <v>44</v>
+        <v>54</v>
+      </c>
+      <c r="I58" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -3869,7 +3866,7 @@
         <v>161</v>
       </c>
       <c r="B59" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D59" t="s">
         <v>41</v>
@@ -3877,8 +3874,11 @@
       <c r="E59" t="s">
         <v>42</v>
       </c>
+      <c r="F59" t="s">
+        <v>35</v>
+      </c>
       <c r="G59" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="H59" t="s">
         <v>44</v>
@@ -3889,16 +3889,19 @@
         <v>161</v>
       </c>
       <c r="B60" t="s">
-        <v>32</v>
+        <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>116</v>
+        <v>41</v>
+      </c>
+      <c r="E60" t="s">
+        <v>42</v>
       </c>
       <c r="G60" t="s">
-        <v>36</v>
+        <v>129</v>
       </c>
       <c r="H60" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -3906,16 +3909,16 @@
         <v>161</v>
       </c>
       <c r="B61" t="s">
-        <v>133</v>
+        <v>32</v>
       </c>
       <c r="D61" t="s">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="G61" t="s">
-        <v>134</v>
+        <v>36</v>
       </c>
       <c r="H61" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3923,13 +3926,13 @@
         <v>161</v>
       </c>
       <c r="B62" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="D62" t="s">
         <v>52</v>
       </c>
       <c r="G62" t="s">
-        <v>35</v>
+        <v>134</v>
       </c>
       <c r="H62" t="s">
         <v>44</v>
@@ -3940,19 +3943,16 @@
         <v>161</v>
       </c>
       <c r="B63" t="s">
-        <v>151</v>
-      </c>
-      <c r="C63" t="s">
-        <v>170</v>
+        <v>111</v>
       </c>
       <c r="D63" t="s">
         <v>52</v>
       </c>
       <c r="G63" t="s">
-        <v>121</v>
+        <v>35</v>
       </c>
       <c r="H63" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3960,19 +3960,19 @@
         <v>161</v>
       </c>
       <c r="B64" t="s">
-        <v>143</v>
+        <v>151</v>
+      </c>
+      <c r="C64" t="s">
+        <v>170</v>
       </c>
       <c r="D64" t="s">
-        <v>75</v>
-      </c>
-      <c r="E64" t="s">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="G64" t="s">
-        <v>171</v>
+        <v>121</v>
       </c>
       <c r="H64" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -3980,13 +3980,16 @@
         <v>161</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="D65" t="s">
-        <v>127</v>
+        <v>75</v>
+      </c>
+      <c r="E65" t="s">
+        <v>82</v>
       </c>
       <c r="G65" t="s">
-        <v>100</v>
+        <v>171</v>
       </c>
       <c r="H65" t="s">
         <v>44</v>
@@ -3997,13 +4000,13 @@
         <v>161</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="D66" t="s">
         <v>127</v>
       </c>
       <c r="G66" t="s">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="H66" t="s">
         <v>44</v>
@@ -4014,13 +4017,13 @@
         <v>161</v>
       </c>
       <c r="B67" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D67" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="G67" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="H67" t="s">
         <v>44</v>
@@ -4031,19 +4034,16 @@
         <v>161</v>
       </c>
       <c r="B68" t="s">
-        <v>63</v>
+        <v>153</v>
       </c>
       <c r="D68" t="s">
-        <v>166</v>
-      </c>
-      <c r="F68" t="s">
-        <v>35</v>
+        <v>52</v>
+      </c>
+      <c r="G68" t="s">
+        <v>87</v>
       </c>
       <c r="H68" t="s">
-        <v>106</v>
-      </c>
-      <c r="K68" t="s">
-        <v>109</v>
+        <v>44</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -4051,16 +4051,19 @@
         <v>161</v>
       </c>
       <c r="B69" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="D69" t="s">
-        <v>52</v>
+        <v>166</v>
+      </c>
+      <c r="F69" t="s">
+        <v>35</v>
       </c>
       <c r="H69" t="s">
         <v>106</v>
       </c>
       <c r="K69" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -4068,19 +4071,16 @@
         <v>161</v>
       </c>
       <c r="B70" t="s">
-        <v>172</v>
+        <v>105</v>
       </c>
       <c r="D70" t="s">
-        <v>41</v>
-      </c>
-      <c r="E70" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H70" t="s">
         <v>106</v>
       </c>
       <c r="K70" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -4088,16 +4088,19 @@
         <v>161</v>
       </c>
       <c r="B71" t="s">
-        <v>115</v>
+        <v>172</v>
       </c>
       <c r="D71" t="s">
-        <v>116</v>
-      </c>
-      <c r="G71" t="s">
-        <v>36</v>
+        <v>41</v>
+      </c>
+      <c r="E71" t="s">
+        <v>42</v>
       </c>
       <c r="H71" t="s">
-        <v>37</v>
+        <v>106</v>
+      </c>
+      <c r="K71" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -4105,7 +4108,7 @@
         <v>161</v>
       </c>
       <c r="B72" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D72" t="s">
         <v>116</v>
@@ -4122,16 +4125,16 @@
         <v>161</v>
       </c>
       <c r="B73" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D73" t="s">
-        <v>52</v>
-      </c>
-      <c r="G73">
-        <v>823</v>
+        <v>116</v>
+      </c>
+      <c r="G73" t="s">
+        <v>36</v>
       </c>
       <c r="H73" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -4139,13 +4142,13 @@
         <v>161</v>
       </c>
       <c r="B74" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D74" t="s">
         <v>52</v>
       </c>
       <c r="G74">
-        <v>-1</v>
+        <v>823</v>
       </c>
       <c r="H74" t="s">
         <v>44</v>
@@ -4156,21 +4159,38 @@
         <v>161</v>
       </c>
       <c r="B75" t="s">
-        <v>158</v>
-      </c>
-      <c r="C75" t="s">
-        <v>173</v>
+        <v>123</v>
       </c>
       <c r="D75" t="s">
         <v>52</v>
       </c>
-      <c r="G75" t="s">
+      <c r="G75">
+        <v>-1</v>
+      </c>
+      <c r="H75" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" t="s">
+        <v>161</v>
+      </c>
+      <c r="B76" t="s">
+        <v>158</v>
+      </c>
+      <c r="C76" t="s">
+        <v>173</v>
+      </c>
+      <c r="D76" t="s">
+        <v>52</v>
+      </c>
+      <c r="G76" t="s">
         <v>174</v>
       </c>
-      <c r="H75" t="s">
+      <c r="H76" t="s">
         <v>54</v>
       </c>
-      <c r="N75" t="s">
+      <c r="N76" t="s">
         <v>175</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: v2.2.21 - sua label mapping DETAIL cho truong Dien tich Son hoan thien trong CK_Mapping_v5.xlsx
- DETAIL R24: "Dien tich (m2) - Son hoan thien" -> "Dien tich (m2) - Son H. Thien"

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tools/config/CK_Mapping_v5.xlsx
+++ b/Tools/config/CK_Mapping_v5.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BOM_Tool\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\insertdatasqlserver\Tools\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6687613-B1E7-41A2-B331-31EB09C546B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B1AEF9-565D-444E-A83A-841CF9699137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1783" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1783" uniqueCount="404">
   <si>
     <t>CK_Mapping_v4 — Sheet 6: HEADER — Mapping đầu phiếu (Section=HEADER → BOM | Section=THDM_HEADER → THDM)</t>
   </si>
@@ -1248,6 +1248,9 @@
   </si>
   <si>
     <t>Hoàn thiện - Số mặt sơn theo mã</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diện tích (m2) - Sơn H. Thiện </t>
   </si>
 </sst>
 </file>
@@ -4808,7 +4811,7 @@
         <v>333</v>
       </c>
       <c r="C24" t="s">
-        <v>334</v>
+        <v>403</v>
       </c>
       <c r="D24" t="s">
         <v>93</v>

</xml_diff>